<commit_message>
Kazanç defteri üreticileri seviye parametreli (SEVIYE=2000/1000/TAM); 2026 Excel 2.000 $
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rzy66tV1hqjtZR3NxuQCPi
</commit_message>
<xml_diff>
--- a/raporlar/kazanc_defteri/Kazanc_2026_Gun_Hafta_Ay.xlsx
+++ b/raporlar/kazanc_defteri/Kazanc_2026_Gun_Hafta_Ay.xlsx
@@ -38,7 +38,7 @@
     <t xml:space="preserve">Kaynak: binance-carry-bot backtest motoru (g33.py), KAR_HARITASI madde 601 / 623 / 628 / 629. Günlük getiriler 'Günlük' sayfasında (mavi = motor çıktısı).</t>
   </si>
   <si>
-    <t xml:space="preserve">Model: gerçekçi (canlı gibi tek hesap girişi + işlem başı 5 bp + düzeltilmiş kademe dolumu), TAM evren (≳ 12.500 $ bakiye), iki dilim hizasının ortalaması.</t>
+    <t xml:space="preserve">Model: gerçekçi (canlı gibi tek hesap girişi + işlem başı 5 bp + düzeltilmiş kademe dolumu), iki dilim hizasının ortalaması. Evren: TAM (≳ 12.500 $ bakiye).</t>
   </si>
   <si>
     <t xml:space="preserve">T4 = kod varsayılanı, kaldıraçsız. T7K 1,15x ve T6 1,10x: günlük getiri × kaldıraç (T4 ile aynı 6 yıllık maks düşüş, madde 596 yöntemi).</t>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Bunlar geçmiş verinin simülasyonudur; canlı hesabın gerçek sonucu değildir ve gelecek için garanti vermez.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 (1 Ocak – 30 Eylül) özet — TAM evren</t>
+    <t xml:space="preserve">2026 (1 Ocak – 30 Eylül) özet — TAM evren (20-100 bin $)</t>
   </si>
   <si>
     <t xml:space="preserve">Ölçü</t>

</xml_diff>